<commit_message>
Pensión total con la reforma (Ley 21.735), GitHub Pages y normalización de líneas
- reforma.py: cotización del empleador a la cuenta individual según fecha, Cotización
  con Rentabilidad Protegida y PGU focalizada. Hallazgo 11, figura 11, hojas Excel
  Pension_total y Pension_por_ingreso, y sección en el tablero.
- Resultado: con supuestos de consenso, la tasa de reemplazo mediana del hombre pasa
  de 27% (solo 10% del trabajador) a 58% con la reforma completa.
- Workflow pages.yml para publicar el tablero y el simulador en GitHub Pages.
- .gitattributes: finales de línea LF en el repositorio.
- 27 pruebas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/reporte_proyecto_afp.xlsx
+++ b/reports/reporte_proyecto_afp.xlsx
@@ -23,8 +23,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bandas_FG" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robustez" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios_mercado" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incertidumbre" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pension_total" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pension_por_ingreso" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incertidumbre" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -532,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -718,6 +720,21 @@
       <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Recentrando los escenarios en el consenso 2026 (renta fija UF 2,52%, renta variable global 4,4% real): Fondo A 4,1% y E 2,7% real/año; ciclo de vida vs por defecto +12% en la mediana (vs +46% con la historia), percentil 5 -2%, gana en 68% de los escenarios. Sin prima de crecimiento: -1%. La probabilidad de alcanzar una tasa de reemplazo de 40% es 10% (por defecto) y 25% (ciclo de vida).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>La reforma de 2025 cambia más la pensión que cualquier estrategia de inversión: la tasa de reemplazo se duplica.</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Fondo por defecto, consenso 2026. Hombre: solo con el 10% del trabajador, tasa de reemplazo mediana 27% (10% llega a 40%); con cotización del empleador, rentabilidad protegida y PGU, 58% (98% llega a 40%). Mujer (PGU desde los 65): 17% → 43%. La PGU es progresiva: con sueldo de 15 UF la tasa total es 69% y con 60 UF, 40%.</t>
         </is>
       </c>
     </row>
@@ -4117,6 +4134,969 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Pensión total con la reforma (Ley 21.735): capas acumuladas, supuestos de consenso 2026 (UF de hoy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>sexo</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>estrategia</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>capa</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>p5</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>mediana</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>tasa_reemplazo_mediana</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>prob_tr_meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Por defecto (ley)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Solo 10% del trabajador</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="n">
+        <v>5.839722702869804</v>
+      </c>
+      <c r="E4" s="25" t="n">
+        <v>9.738421898722411</v>
+      </c>
+      <c r="F4" s="25" t="n">
+        <v>16.28288792490609</v>
+      </c>
+      <c r="G4" s="22" t="n">
+        <v>0.2684710866925683</v>
+      </c>
+      <c r="H4" s="22" t="n">
+        <v>0.1022</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Por defecto (ley)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>+ cotización del empleador</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="n">
+        <v>8.418152002302595</v>
+      </c>
+      <c r="E5" s="25" t="n">
+        <v>13.81534286761175</v>
+      </c>
+      <c r="F5" s="25" t="n">
+        <v>22.63814266675169</v>
+      </c>
+      <c r="G5" s="22" t="n">
+        <v>0.380864595031022</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <v>0.4374</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Por defecto (ley)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>+ rentabilidad protegida</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>9.183865868763188</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>14.58105673407234</v>
+      </c>
+      <c r="F6" s="25" t="n">
+        <v>23.40385653321228</v>
+      </c>
+      <c r="G6" s="22" t="n">
+        <v>0.4019739735280877</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <v>0.5062</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Por defecto (ley)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>+ PGU (pensión total)</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="n">
+        <v>15.4874663070117</v>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>20.88465717232086</v>
+      </c>
+      <c r="F7" s="25" t="n">
+        <v>27.80227090998295</v>
+      </c>
+      <c r="G7" s="22" t="n">
+        <v>0.5757531009198006</v>
+      </c>
+      <c r="H7" s="22" t="n">
+        <v>0.9798</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Ciclo de vida (aprox. FG)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Solo 10% del trabajador</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>5.699918912448215</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>10.89820160052584</v>
+      </c>
+      <c r="F8" s="25" t="n">
+        <v>22.7324423449607</v>
+      </c>
+      <c r="G8" s="22" t="n">
+        <v>0.3004441640664289</v>
+      </c>
+      <c r="H8" s="22" t="n">
+        <v>0.2542</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Ciclo de vida (aprox. FG)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>+ cotización del empleador</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>8.292079938934828</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>15.31046702704942</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>30.8519879078192</v>
+      </c>
+      <c r="G9" s="22" t="n">
+        <v>0.4220825266424266</v>
+      </c>
+      <c r="H9" s="22" t="n">
+        <v>0.5534</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Ciclo de vida (aprox. FG)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>+ rentabilidad protegida</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>9.057793805395422</v>
+      </c>
+      <c r="E10" s="25" t="n">
+        <v>16.07618089351001</v>
+      </c>
+      <c r="F10" s="25" t="n">
+        <v>31.6177017742798</v>
+      </c>
+      <c r="G10" s="22" t="n">
+        <v>0.4431919051394922</v>
+      </c>
+      <c r="H10" s="22" t="n">
+        <v>0.6065</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Ciclo de vida (aprox. FG)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>+ PGU (pensión total)</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>15.36139424364394</v>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>22.37978133175853</v>
+      </c>
+      <c r="F11" s="25" t="n">
+        <v>31.6177017742798</v>
+      </c>
+      <c r="G11" s="22" t="n">
+        <v>0.6169710325312051</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <v>0.9766</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Por defecto (ley)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Solo 10% del trabajador</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>3.885048758221369</v>
+      </c>
+      <c r="E12" s="25" t="n">
+        <v>6.299769863417148</v>
+      </c>
+      <c r="F12" s="25" t="n">
+        <v>10.07880475761453</v>
+      </c>
+      <c r="G12" s="22" t="n">
+        <v>0.1736735252111615</v>
+      </c>
+      <c r="H12" s="22" t="n">
+        <v>0.0009</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Por defecto (ley)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>+ cotización del empleador</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="n">
+        <v>5.55684712339447</v>
+      </c>
+      <c r="E13" s="25" t="n">
+        <v>8.847044098554148</v>
+      </c>
+      <c r="F13" s="25" t="n">
+        <v>13.85461057598768</v>
+      </c>
+      <c r="G13" s="22" t="n">
+        <v>0.2438973755560442</v>
+      </c>
+      <c r="H13" s="22" t="n">
+        <v>0.0335</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Por defecto (ley)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>+ rentabilidad protegida</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="n">
+        <v>6.117704471929141</v>
+      </c>
+      <c r="E14" s="25" t="n">
+        <v>9.40790144708882</v>
+      </c>
+      <c r="F14" s="25" t="n">
+        <v>14.41546792452235</v>
+      </c>
+      <c r="G14" s="22" t="n">
+        <v>0.2593592217777991</v>
+      </c>
+      <c r="H14" s="22" t="n">
+        <v>0.0475</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Por defecto (ley)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>+ PGU (pensión total)</t>
+        </is>
+      </c>
+      <c r="D15" s="25" t="n">
+        <v>12.42130491017766</v>
+      </c>
+      <c r="E15" s="25" t="n">
+        <v>15.71150188533734</v>
+      </c>
+      <c r="F15" s="25" t="n">
+        <v>20.71906836277087</v>
+      </c>
+      <c r="G15" s="22" t="n">
+        <v>0.433138349169512</v>
+      </c>
+      <c r="H15" s="22" t="n">
+        <v>0.6962</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Ciclo de vida (aprox. FG)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Solo 10% del trabajador</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="n">
+        <v>3.692104512885175</v>
+      </c>
+      <c r="E16" s="25" t="n">
+        <v>7.141355359638041</v>
+      </c>
+      <c r="F16" s="25" t="n">
+        <v>14.78860243300412</v>
+      </c>
+      <c r="G16" s="22" t="n">
+        <v>0.1968745504968671</v>
+      </c>
+      <c r="H16" s="22" t="n">
+        <v>0.0544</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Ciclo de vida (aprox. FG)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>+ cotización del empleador</t>
+        </is>
+      </c>
+      <c r="D17" s="25" t="n">
+        <v>5.3167074723396</v>
+      </c>
+      <c r="E17" s="25" t="n">
+        <v>9.933573226557268</v>
+      </c>
+      <c r="F17" s="25" t="n">
+        <v>19.90311772943648</v>
+      </c>
+      <c r="G17" s="22" t="n">
+        <v>0.2738510640234123</v>
+      </c>
+      <c r="H17" s="22" t="n">
+        <v>0.1787</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Ciclo de vida (aprox. FG)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>+ rentabilidad protegida</t>
+        </is>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>5.87756482087427</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>10.49443057509194</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>20.46397507797115</v>
+      </c>
+      <c r="G18" s="22" t="n">
+        <v>0.2893129102451671</v>
+      </c>
+      <c r="H18" s="22" t="n">
+        <v>0.2064</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Ciclo de vida (aprox. FG)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>+ PGU (pensión total)</t>
+        </is>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>12.18116525912279</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>16.79803101334046</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>26.44995703016958</v>
+      </c>
+      <c r="G19" s="22" t="n">
+        <v>0.4630920376368801</v>
+      </c>
+      <c r="H19" s="22" t="n">
+        <v>0.7491</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Capas: 10% del trabajador; + cotización del empleador a la cuenta individual (0,1% → 6% según fecha); + Cotización con Rentabilidad Protegida (bono a 2,52% real); + PGU ($250.275 feb-2026, focalizada por pensión base).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Mujer: se pensiona a los 60 y recibe la PGU desde los 65. Supone que cumple la focalización (no es del 10% más rico).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Tasa de reemplazo = pensión / último sueldo imponible. Meta: 40%.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Progresividad: pensión total mediana por nivel de sueldo (fondo por defecto, consenso 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>sueldo_inicial_uf</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>sueldo_final_uf</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>autofinanciada_10</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>empleador_cci</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>crp</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>pgu</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>tasa_reemplazo_total</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>tasa_reemplazo_10</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>sexo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="B4" s="25" t="n">
+        <v>21.76418031161935</v>
+      </c>
+      <c r="C4" s="25" t="n">
+        <v>5.786789754691971</v>
+      </c>
+      <c r="D4" s="25" t="n">
+        <v>2.501554667283413</v>
+      </c>
+      <c r="E4" s="25" t="n">
+        <v>0.4594283198763565</v>
+      </c>
+      <c r="F4" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="G4" s="25" t="n">
+        <v>15.05137318010026</v>
+      </c>
+      <c r="H4" s="22" t="n">
+        <v>0.6915662783801099</v>
+      </c>
+      <c r="I4" s="22" t="n">
+        <v>0.2658859498422069</v>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="B5" s="25" t="n">
+        <v>36.27363385269892</v>
+      </c>
+      <c r="C5" s="25" t="n">
+        <v>9.644649591153307</v>
+      </c>
+      <c r="D5" s="25" t="n">
+        <v>4.16925777880572</v>
+      </c>
+      <c r="E5" s="25" t="n">
+        <v>0.765713866460594</v>
+      </c>
+      <c r="F5" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="G5" s="25" t="n">
+        <v>20.88322167466814</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <v>0.5757135267856361</v>
+      </c>
+      <c r="I5" s="22" t="n">
+        <v>0.2658859498422075</v>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="B6" s="25" t="n">
+        <v>58.03781416431828</v>
+      </c>
+      <c r="C6" s="25" t="n">
+        <v>15.66654838500849</v>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>6.440296999414378</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>1.22514218633695</v>
+      </c>
+      <c r="F6" s="25" t="n">
+        <v>4.437224388740966</v>
+      </c>
+      <c r="G6" s="25" t="n">
+        <v>27.76921195950079</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <v>0.4784675708302835</v>
+      </c>
+      <c r="I6" s="22" t="n">
+        <v>0.2699369128660312</v>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="B7" s="25" t="n">
+        <v>87.05672124647741</v>
+      </c>
+      <c r="C7" s="25" t="n">
+        <v>23.49982257751299</v>
+      </c>
+      <c r="D7" s="25" t="n">
+        <v>9.660445499121563</v>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>1.837713279505426</v>
+      </c>
+      <c r="F7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="25" t="n">
+        <v>34.99798135613999</v>
+      </c>
+      <c r="H7" s="22" t="n">
+        <v>0.4020135476622503</v>
+      </c>
+      <c r="I7" s="22" t="n">
+        <v>0.2699369128660341</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="B8" s="25" t="n">
+        <v>21.76418031161935</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <v>3.763768244189001</v>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>1.544055219449044</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>0.3365144091208025</v>
+      </c>
+      <c r="F8" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="G8" s="25" t="n">
+        <v>11.94793831100736</v>
+      </c>
+      <c r="H8" s="22" t="n">
+        <v>0.5489725843076505</v>
+      </c>
+      <c r="I8" s="22" t="n">
+        <v>0.1729340682855682</v>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="B9" s="25" t="n">
+        <v>36.27363385269892</v>
+      </c>
+      <c r="C9" s="25" t="n">
+        <v>6.272947073648333</v>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>2.573425365748407</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>0.5608573485346711</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="G9" s="25" t="n">
+        <v>15.71083022617993</v>
+      </c>
+      <c r="H9" s="22" t="n">
+        <v>0.4331198327131753</v>
+      </c>
+      <c r="I9" s="22" t="n">
+        <v>0.1729340682855682</v>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="B10" s="25" t="n">
+        <v>58.03781416431828</v>
+      </c>
+      <c r="C10" s="25" t="n">
+        <v>9.960261600228364</v>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>4.196083612110052</v>
+      </c>
+      <c r="E10" s="25" t="n">
+        <v>0.8973717576554735</v>
+      </c>
+      <c r="F10" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="G10" s="25" t="n">
+        <v>21.35731740824241</v>
+      </c>
+      <c r="H10" s="22" t="n">
+        <v>0.3679896928539551</v>
+      </c>
+      <c r="I10" s="22" t="n">
+        <v>0.1716167595841669</v>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="B11" s="25" t="n">
+        <v>87.05672124647741</v>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>15.055072976756</v>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>6.176220877796176</v>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>1.34605763648321</v>
+      </c>
+      <c r="F11" s="25" t="n">
+        <v>4.844735980503486</v>
+      </c>
+      <c r="G11" s="25" t="n">
+        <v>27.42208747153887</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <v>0.3149910435278248</v>
+      </c>
+      <c r="I11" s="22" t="n">
+        <v>0.1729340682855682</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5679,93 +6659,6 @@
       <c r="A65" s="2" t="inlineStr">
         <is>
           <t>GARCH: simulación histórica filtrada (residuos estandarizados remuestreados). Persistencia 0,9999 = tope de la restricción (volatilidad integrada, vida media no acotada).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="140" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Valores cuota y patrimonio: Superintendencia de Pensiones, spensiones.cl/apps/valoresCuotaFondo/vcfAFP.php (2002-2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Afiliados por edad y AFP: SP, Series estadísticas del Sistema de Pensiones (trimestral).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Tablas de mortalidad CB-H-2020 y RV-M-2020: CMF, NCG N.º 495 (feb-2023).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>TITRP 3,45%: SP, Circular N.º 2417 (07-07-2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>UF diaria: Banco Central de Chile, Base de Datos Estadísticos (API SieteRestWS).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Régimen de inversión de los Fondos Generacionales: SP, Res. Ex. N.º 1195 (01-09-2026); bandas de 240 a 290 p.b. anuales, transición de 400 p.b. entre abr-2028 y mar-2031 (spensiones.cl/portal/institucional/594/w3-article-17131.html).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Trayectoria de inversión (máximo de activos de crecimiento por edad): SP, minuta de la consulta pública (jul-2026, articles-11315_nt_561_minuta.pdf), digitalizada; tope inicial de 95% de la versión definitiva (Res. Ex. N.º 1195).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Activos de crecimiento de cada multifondo: SP, Reporte mensual de inversiones, cartera al 31-03-2026 (tablas 16 y 18).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Renta fija en UF: tasa de bonos BCU/BTU a 10 años, mercado secundario, 2,52% (BCCh, 08-06-2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Renta variable global: MSCI ACWI 7,0% nominal USD e inflación EE.UU. 2,5% (J.P. Morgan AM, Long-Term Capital Market Assumptions 2026).</t>
         </is>
       </c>
     </row>
@@ -29690,6 +30583,100 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="140" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Valores cuota y patrimonio: Superintendencia de Pensiones, spensiones.cl/apps/valoresCuotaFondo/vcfAFP.php (2002-2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Afiliados por edad y AFP: SP, Series estadísticas del Sistema de Pensiones (trimestral).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Tablas de mortalidad CB-H-2020 y RV-M-2020: CMF, NCG N.º 495 (feb-2023).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>TITRP 3,45%: SP, Circular N.º 2417 (07-07-2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>UF diaria: Banco Central de Chile, Base de Datos Estadísticos (API SieteRestWS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Régimen de inversión de los Fondos Generacionales: SP, Res. Ex. N.º 1195 (01-09-2026); bandas de 240 a 290 p.b. anuales, transición de 400 p.b. entre abr-2028 y mar-2031 (spensiones.cl/portal/institucional/594/w3-article-17131.html).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Trayectoria de inversión (máximo de activos de crecimiento por edad): SP, minuta de la consulta pública (jul-2026, articles-11315_nt_561_minuta.pdf), digitalizada; tope inicial de 95% de la versión definitiva (Res. Ex. N.º 1195).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Activos de crecimiento de cada multifondo: SP, Reporte mensual de inversiones, cartera al 31-03-2026 (tablas 16 y 18).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Renta fija en UF: tasa de bonos BCU/BTU a 10 años, mercado secundario, 2,52% (BCCh, 08-06-2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Renta variable global: MSCI ACWI 7,0% nominal USD e inflación EE.UU. 2,5% (J.P. Morgan AM, Long-Term Capital Market Assumptions 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Reforma de pensiones: Ley N.º 21.735; Subsecretaría de Previsión Social, Nota Técnica (ago-2025), tablas 1, 3 y 5. PGU y umbrales de pensión base: SP (vigentes desde el 01-02-2026).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Glidepath óptimo por utilidad CRRA de la pensión total
- optimo.py: busca el mejor glidepath de la familia "meseta y bajada" maximizando el
  equivalente cierto CRRA (gamma 2, 3 y 5), con y sin la reforma, con escenarios de
  entrenamiento y prueba separados y ejecución en paralelo.
- Resultado: el glidepath oficial queda a 0,3%-3,1% del óptimo; la ley por defecto,
  1%-9% bajo el oficial. Con la PGU, el óptimo llega al retiro con más riesgo (70% vs 40%).
- Hallazgo 12, figura 12, hoja Excel Glidepath_optimo, línea en el tablero.
- Salida gzip reproducible (sin marca de tiempo). 29 pruebas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/reporte_proyecto_afp.xlsx
+++ b/reports/reporte_proyecto_afp.xlsx
@@ -25,8 +25,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios_mercado" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pension_total" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pension_por_ingreso" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incertidumbre" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glidepath_optimo" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incertidumbre" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -534,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -735,6 +736,21 @@
       <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Fondo por defecto, consenso 2026. Hombre: solo con el 10% del trabajador, tasa de reemplazo mediana 27% (10% llega a 40%); con cotización del empleador, rentabilidad protegida y PGU, 58% (98% llega a 40%). Mujer (PGU desde los 65): 17% → 43%. La PGU es progresiva: con sueldo de 15 UF la tasa total es 69% y con 60 UF, 40%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>El glidepath oficial está muy cerca del óptimo, y la PGU justifica llegar al retiro con más riesgo.</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Maximizando la utilidad CRRA de la pensión total (hombre, consenso 2026, escenarios de prueba), el mejor glidepath de la familia supera al oficial en solo +0,3% a +3,1% de pensión equivalente cierta (aversión γ de 2 a 5); el fondo por defecto de la ley queda -9% a -1% bajo el oficial. Con γ = 3, el óptimo llega al retiro con 70% en crecimiento si se cuenta la PGU y 40% sin ella (el oficial, 29%): la PGU actúa como un bono.</t>
         </is>
       </c>
     </row>
@@ -5097,1568 +5113,326 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>Incertidumbre de parámetros: intervalos de confianza de 90% por bootstrap (percentiles 5–95)</t>
+          <t>¿Es óptimo el glidepath oficial? Mejor glidepath de la familia por aversión al riesgo (equivalente cierto, UF)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>bloque</t>
+          <t>sexo</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>regimen</t>
+          <t>gamma</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>fondo</t>
+          <t>con_reforma</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>metrica</t>
+          <t>g0</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>p05</t>
+          <t>a1</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>mediana</t>
+          <t>g1</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>ec_oficial</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>ec_optimo</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>ec_defecto</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>optimo_vs_oficial</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>defecto_vs_oficial</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Pensiones (historia remuestreada)</t>
+          <t>H</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>prima_real_A_vs_E</t>
-        </is>
-      </c>
-      <c r="E4" s="24" t="n">
-        <v>-0.02033327831223074</v>
-      </c>
-      <c r="F4" s="24" t="n">
-        <v>0.03465617575860558</v>
-      </c>
-      <c r="G4" s="24" t="n">
-        <v>0.07218940162832164</v>
+      <c r="B4" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="27" t="n">
+        <v>45</v>
+      </c>
+      <c r="F4" s="22" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G4" s="25" t="n">
+        <v>21.81089144260766</v>
+      </c>
+      <c r="H4" s="25" t="n">
+        <v>22.49791750733205</v>
+      </c>
+      <c r="I4" s="25" t="n">
+        <v>20.54633424268781</v>
+      </c>
+      <c r="J4" s="22" t="n">
+        <v>0.03149921985225612</v>
+      </c>
+      <c r="K4" s="22" t="n">
+        <v>-0.05797824464201073</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Pensiones (historia remuestreada)</t>
+          <t>H</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>cv_vs_defecto_mediana</t>
-        </is>
-      </c>
-      <c r="E5" s="24" t="n">
-        <v>-0.1414839611704128</v>
-      </c>
-      <c r="F5" s="24" t="n">
-        <v>0.3976446313068648</v>
-      </c>
-      <c r="G5" s="24" t="n">
-        <v>1.19503782136728</v>
+      <c r="B5" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="27" t="n">
+        <v>35</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G5" s="25" t="n">
+        <v>21.24106514110735</v>
+      </c>
+      <c r="H5" s="25" t="n">
+        <v>21.47962732253391</v>
+      </c>
+      <c r="I5" s="25" t="n">
+        <v>20.20551993500472</v>
+      </c>
+      <c r="J5" s="22" t="n">
+        <v>0.01123117790194428</v>
+      </c>
+      <c r="K5" s="22" t="n">
+        <v>-0.04875203758490254</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Pensiones (historia remuestreada)</t>
+          <t>H</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>cv_vs_defecto_p5</t>
-        </is>
-      </c>
-      <c r="E6" s="24" t="n">
-        <v>-0.2811320009079319</v>
-      </c>
-      <c r="F6" s="24" t="n">
-        <v>0.07979349629326404</v>
-      </c>
-      <c r="G6" s="24" t="n">
-        <v>0.6815268945114384</v>
+      <c r="B6" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G6" s="25" t="n">
+        <v>20.21040530232428</v>
+      </c>
+      <c r="H6" s="25" t="n">
+        <v>20.27355184298723</v>
+      </c>
+      <c r="I6" s="25" t="n">
+        <v>19.55520649790904</v>
+      </c>
+      <c r="J6" s="22" t="n">
+        <v>0.003124456918025542</v>
+      </c>
+      <c r="K6" s="22" t="n">
+        <v>-0.03241888495625012</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Pensiones (historia remuestreada)</t>
+          <t>H</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>prob_cv_supera_defecto</t>
-        </is>
-      </c>
-      <c r="E7" s="24" t="n">
-        <v>0.22735</v>
-      </c>
-      <c r="F7" s="24" t="n">
-        <v>0.92075</v>
-      </c>
-      <c r="G7" s="24" t="n">
-        <v>0.999525</v>
+      <c r="B7" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <v>35</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G7" s="25" t="n">
+        <v>10.15941939138435</v>
+      </c>
+      <c r="H7" s="25" t="n">
+        <v>10.37332862672469</v>
+      </c>
+      <c r="I7" s="25" t="n">
+        <v>9.263241171699766</v>
+      </c>
+      <c r="J7" s="22" t="n">
+        <v>0.02105526183137507</v>
+      </c>
+      <c r="K7" s="22" t="n">
+        <v>-0.08821155866885277</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Pensiones (historia remuestreada)</t>
+          <t>H</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>reactivo_vs_defecto_mediana</t>
-        </is>
-      </c>
-      <c r="E8" s="24" t="n">
-        <v>-0.08690068468870106</v>
-      </c>
-      <c r="F8" s="24" t="n">
-        <v>-0.03463701503838251</v>
-      </c>
-      <c r="G8" s="24" t="n">
-        <v>0.08547595265559825</v>
+      <c r="B8" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G8" s="25" t="n">
+        <v>9.379509959857522</v>
+      </c>
+      <c r="H8" s="25" t="n">
+        <v>9.434561713195848</v>
+      </c>
+      <c r="I8" s="25" t="n">
+        <v>8.826324808747481</v>
+      </c>
+      <c r="J8" s="22" t="n">
+        <v>0.005869363492755575</v>
+      </c>
+      <c r="K8" s="22" t="n">
+        <v>-0.0589780439999068</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Pensiones (historia remuestreada)</t>
+          <t>H</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="B9" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G9" s="25" t="n">
+        <v>8.093007015597816</v>
+      </c>
+      <c r="H9" s="25" t="n">
+        <v>8.29561118747621</v>
+      </c>
+      <c r="I9" s="25" t="n">
+        <v>8.025854067417487</v>
+      </c>
+      <c r="J9" s="22" t="n">
+        <v>0.02503447377321066</v>
+      </c>
+      <c r="K9" s="22" t="n">
+        <v>-0.008297651052433741</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>mediana_defecto_uf</t>
+          <t>Familia: meseta g0 hasta la edad a1 y baja lineal hasta g1 al retiro; réplica con multifondos.</t>
         </is>
       </c>
-      <c r="E9" s="24" t="n">
-        <v>6.425983355851145</v>
-      </c>
-      <c r="F9" s="24" t="n">
-        <v>10.94096361298217</v>
-      </c>
-      <c r="G9" s="24" t="n">
-        <v>18.88060876426169</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HMM (paramétrico)</t>
+          <t>Criterio: utilidad CRRA de la pensión total (con_reforma = cotización del empleador, rentabilidad protegida y PGU).</t>
         </is>
       </c>
-      <c r="B10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="inlineStr">
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>persistencia</t>
-        </is>
-      </c>
-      <c r="E10" s="24" t="n">
-        <v>0.89955905324987</v>
-      </c>
-      <c r="F10" s="24" t="n">
-        <v>0.9501451205084048</v>
-      </c>
-      <c r="G10" s="24" t="n">
-        <v>0.9784178788593505</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>persistencia</t>
-        </is>
-      </c>
-      <c r="E11" s="24" t="n">
-        <v>0.6474081362214877</v>
-      </c>
-      <c r="F11" s="24" t="n">
-        <v>0.9833498083623404</v>
-      </c>
-      <c r="G11" s="24" t="n">
-        <v>0.9999999999978014</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>persistencia</t>
-        </is>
-      </c>
-      <c r="E12" s="24" t="n">
-        <v>0.2660517766209279</v>
-      </c>
-      <c r="F12" s="24" t="n">
-        <v>0.583671287299481</v>
-      </c>
-      <c r="G12" s="24" t="n">
-        <v>0.7756626825602544</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>duracion_meses</t>
-        </is>
-      </c>
-      <c r="E13" s="24" t="n">
-        <v>9.957652483720244</v>
-      </c>
-      <c r="F13" s="24" t="n">
-        <v>20.05835072661364</v>
-      </c>
-      <c r="G13" s="24" t="n">
-        <v>46.33960453807429</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>duracion_meses</t>
-        </is>
-      </c>
-      <c r="E14" s="24" t="n">
-        <v>2.837891664061405</v>
-      </c>
-      <c r="F14" s="24" t="n">
-        <v>60.09146038435532</v>
-      </c>
-      <c r="G14" s="24" t="n">
-        <v>454864035038.6853</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>duracion_meses</t>
-        </is>
-      </c>
-      <c r="E15" s="24" t="n">
-        <v>1.362495000031719</v>
-      </c>
-      <c r="F15" s="24" t="n">
-        <v>2.401949922421466</v>
-      </c>
-      <c r="G15" s="24" t="n">
-        <v>4.45763134079152</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>prob_estacionaria</t>
-        </is>
-      </c>
-      <c r="E16" s="24" t="n">
-        <v>3.910517304810142e-10</v>
-      </c>
-      <c r="F16" s="24" t="n">
-        <v>0.4847451207069491</v>
-      </c>
-      <c r="G16" s="24" t="n">
-        <v>0.8871964979924858</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>prob_estacionaria</t>
-        </is>
-      </c>
-      <c r="E17" s="24" t="n">
-        <v>0.0322741205452757</v>
-      </c>
-      <c r="F17" s="24" t="n">
-        <v>0.4256052965692377</v>
-      </c>
-      <c r="G17" s="24" t="n">
-        <v>0.9999999995623813</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>prob_estacionaria</t>
-        </is>
-      </c>
-      <c r="E18" s="24" t="n">
-        <v>3.683308530043981e-11</v>
-      </c>
-      <c r="F18" s="24" t="n">
-        <v>0.06387070500183775</v>
-      </c>
-      <c r="G18" s="24" t="n">
-        <v>0.1363100918200183</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>vol_A</t>
-        </is>
-      </c>
-      <c r="E19" s="24" t="n">
-        <v>0.08072897392403221</v>
-      </c>
-      <c r="F19" s="24" t="n">
-        <v>0.09235118502937775</v>
-      </c>
-      <c r="G19" s="24" t="n">
-        <v>0.1032374440937383</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>vol_A</t>
-        </is>
-      </c>
-      <c r="E20" s="24" t="n">
-        <v>0.08364058419755244</v>
-      </c>
-      <c r="F20" s="24" t="n">
-        <v>0.09981075731458454</v>
-      </c>
-      <c r="G20" s="24" t="n">
-        <v>0.1162739099861504</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>vol_A</t>
-        </is>
-      </c>
-      <c r="E21" s="24" t="n">
-        <v>0.1564126355374283</v>
-      </c>
-      <c r="F21" s="24" t="n">
-        <v>0.2530674011517392</v>
-      </c>
-      <c r="G21" s="24" t="n">
-        <v>0.3329043933475438</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B22" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>vol_B</t>
-        </is>
-      </c>
-      <c r="E22" s="24" t="n">
-        <v>0.06005314301343295</v>
-      </c>
-      <c r="F22" s="24" t="n">
-        <v>0.06867665571737128</v>
-      </c>
-      <c r="G22" s="24" t="n">
-        <v>0.07771607927689948</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>vol_B</t>
-        </is>
-      </c>
-      <c r="E23" s="24" t="n">
-        <v>0.0687710602341676</v>
-      </c>
-      <c r="F23" s="24" t="n">
-        <v>0.08079676866842468</v>
-      </c>
-      <c r="G23" s="24" t="n">
-        <v>0.09261084260112568</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>vol_B</t>
-        </is>
-      </c>
-      <c r="E24" s="24" t="n">
-        <v>0.1154395579469629</v>
-      </c>
-      <c r="F24" s="24" t="n">
-        <v>0.1828913218922641</v>
-      </c>
-      <c r="G24" s="24" t="n">
-        <v>0.2428672856036235</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>vol_C</t>
-        </is>
-      </c>
-      <c r="E25" s="24" t="n">
-        <v>0.04326168969124074</v>
-      </c>
-      <c r="F25" s="24" t="n">
-        <v>0.04878185657965282</v>
-      </c>
-      <c r="G25" s="24" t="n">
-        <v>0.05514623373205125</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B26" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>vol_C</t>
-        </is>
-      </c>
-      <c r="E26" s="24" t="n">
-        <v>0.05935831197621191</v>
-      </c>
-      <c r="F26" s="24" t="n">
-        <v>0.07051952792886923</v>
-      </c>
-      <c r="G26" s="24" t="n">
-        <v>0.08185603289511963</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B27" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>vol_C</t>
-        </is>
-      </c>
-      <c r="E27" s="24" t="n">
-        <v>0.0783586503246361</v>
-      </c>
-      <c r="F27" s="24" t="n">
-        <v>0.1262760922522181</v>
-      </c>
-      <c r="G27" s="24" t="n">
-        <v>0.164751908648498</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B28" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>vol_D</t>
-        </is>
-      </c>
-      <c r="E28" s="24" t="n">
-        <v>0.02729406917385757</v>
-      </c>
-      <c r="F28" s="24" t="n">
-        <v>0.0313933118895233</v>
-      </c>
-      <c r="G28" s="24" t="n">
-        <v>0.0359455172190928</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>vol_D</t>
-        </is>
-      </c>
-      <c r="E29" s="24" t="n">
-        <v>0.05929960760715521</v>
-      </c>
-      <c r="F29" s="24" t="n">
-        <v>0.07988590968454415</v>
-      </c>
-      <c r="G29" s="24" t="n">
-        <v>0.09224665384603417</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>vol_D</t>
-        </is>
-      </c>
-      <c r="E30" s="24" t="n">
-        <v>0.06581503427343903</v>
-      </c>
-      <c r="F30" s="24" t="n">
-        <v>0.09200615930554423</v>
-      </c>
-      <c r="G30" s="24" t="n">
-        <v>0.1203053956782151</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B31" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>vol_E</t>
-        </is>
-      </c>
-      <c r="E31" s="24" t="n">
-        <v>0.02153802834504729</v>
-      </c>
-      <c r="F31" s="24" t="n">
-        <v>0.02444829465876444</v>
-      </c>
-      <c r="G31" s="24" t="n">
-        <v>0.02714313140970778</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B32" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>vol_E</t>
-        </is>
-      </c>
-      <c r="E32" s="24" t="n">
-        <v>0.05854130433802626</v>
-      </c>
-      <c r="F32" s="24" t="n">
-        <v>0.08849692842917048</v>
-      </c>
-      <c r="G32" s="24" t="n">
-        <v>0.1022842599529493</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B33" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>vol_E</t>
-        </is>
-      </c>
-      <c r="E33" s="24" t="n">
-        <v>0.04960653960172515</v>
-      </c>
-      <c r="F33" s="24" t="n">
-        <v>0.07487598553830438</v>
-      </c>
-      <c r="G33" s="24" t="n">
-        <v>0.09562749248288493</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B34" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>pct_meses_reg1_desde_quiebre</t>
-        </is>
-      </c>
-      <c r="E34" s="24" t="n">
-        <v>0.2823863636363637</v>
-      </c>
-      <c r="F34" s="24" t="n">
-        <v>0.9090909090909091</v>
-      </c>
-      <c r="G34" s="24" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B35" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>pct_meses_reg1_desde_quiebre</t>
-        </is>
-      </c>
-      <c r="E35" s="24" t="n">
-        <v>0.2823863636363637</v>
-      </c>
-      <c r="F35" s="24" t="n">
-        <v>0.9090909090909091</v>
-      </c>
-      <c r="G35" s="24" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>HMM (paramétrico)</t>
-        </is>
-      </c>
-      <c r="B36" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>pct_meses_reg1_desde_quiebre</t>
-        </is>
-      </c>
-      <c r="E36" s="24" t="n">
-        <v>0.2823863636363637</v>
-      </c>
-      <c r="F36" s="24" t="n">
-        <v>0.9090909090909091</v>
-      </c>
-      <c r="G36" s="24" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>alpha</t>
-        </is>
-      </c>
-      <c r="E37" s="24" t="n">
-        <v>0.07144614325844531</v>
-      </c>
-      <c r="F37" s="24" t="n">
-        <v>0.08754058087794941</v>
-      </c>
-      <c r="G37" s="24" t="n">
-        <v>0.1047518854535187</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>alpha</t>
-        </is>
-      </c>
-      <c r="E38" s="24" t="n">
-        <v>0.07088467206040881</v>
-      </c>
-      <c r="F38" s="24" t="n">
-        <v>0.08319216147796728</v>
-      </c>
-      <c r="G38" s="24" t="n">
-        <v>0.09794931987327024</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="n"/>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>alpha</t>
-        </is>
-      </c>
-      <c r="E39" s="24" t="n">
-        <v>0.07743559641469437</v>
-      </c>
-      <c r="F39" s="24" t="n">
-        <v>0.09323644048369883</v>
-      </c>
-      <c r="G39" s="24" t="n">
-        <v>0.1064908875409975</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>alpha</t>
-        </is>
-      </c>
-      <c r="E40" s="24" t="n">
-        <v>0.1014273304397348</v>
-      </c>
-      <c r="F40" s="24" t="n">
-        <v>0.1229886920436335</v>
-      </c>
-      <c r="G40" s="24" t="n">
-        <v>0.1458810224153635</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>alpha</t>
-        </is>
-      </c>
-      <c r="E41" s="24" t="n">
-        <v>0.08009149425301412</v>
-      </c>
-      <c r="F41" s="24" t="n">
-        <v>0.0962849069734741</v>
-      </c>
-      <c r="G41" s="24" t="n">
-        <v>0.1147972241326145</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="n"/>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>beta</t>
-        </is>
-      </c>
-      <c r="E42" s="24" t="n">
-        <v>0.870869662087573</v>
-      </c>
-      <c r="F42" s="24" t="n">
-        <v>0.8901119225657519</v>
-      </c>
-      <c r="G42" s="24" t="n">
-        <v>0.9087228392715047</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>beta</t>
-        </is>
-      </c>
-      <c r="E43" s="24" t="n">
-        <v>0.8847315189449467</v>
-      </c>
-      <c r="F43" s="24" t="n">
-        <v>0.9005922259810597</v>
-      </c>
-      <c r="G43" s="24" t="n">
-        <v>0.9158012795043712</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>beta</t>
-        </is>
-      </c>
-      <c r="E44" s="24" t="n">
-        <v>0.8732655999838247</v>
-      </c>
-      <c r="F44" s="24" t="n">
-        <v>0.8916758752359082</v>
-      </c>
-      <c r="G44" s="24" t="n">
-        <v>0.9107327299916633</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>beta</t>
-        </is>
-      </c>
-      <c r="E45" s="24" t="n">
-        <v>0.8540189775846361</v>
-      </c>
-      <c r="F45" s="24" t="n">
-        <v>0.8744521527367413</v>
-      </c>
-      <c r="G45" s="24" t="n">
-        <v>0.8905375360706199</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="n"/>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>beta</t>
-        </is>
-      </c>
-      <c r="E46" s="24" t="n">
-        <v>0.8808514806269054</v>
-      </c>
-      <c r="F46" s="24" t="n">
-        <v>0.9015989580759767</v>
-      </c>
-      <c r="G46" s="24" t="n">
-        <v>0.9149080365003966</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>persistencia</t>
-        </is>
-      </c>
-      <c r="E47" s="24" t="n">
-        <v>0.9670784595380398</v>
-      </c>
-      <c r="F47" s="24" t="n">
-        <v>0.9792250356075567</v>
-      </c>
-      <c r="G47" s="24" t="n">
-        <v>0.9868330247899996</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="n"/>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>persistencia</t>
-        </is>
-      </c>
-      <c r="E48" s="24" t="n">
-        <v>0.9762799801440459</v>
-      </c>
-      <c r="F48" s="24" t="n">
-        <v>0.9850554519333534</v>
-      </c>
-      <c r="G48" s="24" t="n">
-        <v>0.9912263501073139</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>persistencia</t>
-        </is>
-      </c>
-      <c r="E49" s="24" t="n">
-        <v>0.9754048323534276</v>
-      </c>
-      <c r="F49" s="24" t="n">
-        <v>0.9841341292347877</v>
-      </c>
-      <c r="G49" s="24" t="n">
-        <v>0.9921234543191135</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="n"/>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>persistencia</t>
-        </is>
-      </c>
-      <c r="E50" s="24" t="n">
-        <v>0.9901176467880164</v>
-      </c>
-      <c r="F50" s="24" t="n">
-        <v>0.9998999999999985</v>
-      </c>
-      <c r="G50" s="24" t="n">
-        <v>0.9998999999999998</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>persistencia</t>
-        </is>
-      </c>
-      <c r="E51" s="24" t="n">
-        <v>0.9841933602805655</v>
-      </c>
-      <c r="F51" s="24" t="n">
-        <v>0.9982613817048831</v>
-      </c>
-      <c r="G51" s="24" t="n">
-        <v>0.9998999999999977</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>vida_media_dias</t>
-        </is>
-      </c>
-      <c r="E52" s="24" t="n">
-        <v>20.70605048140716</v>
-      </c>
-      <c r="F52" s="24" t="n">
-        <v>33.01688513161351</v>
-      </c>
-      <c r="G52" s="24" t="n">
-        <v>52.29661231461255</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>vida_media_dias</t>
-        </is>
-      </c>
-      <c r="E53" s="24" t="n">
-        <v>28.87553394898189</v>
-      </c>
-      <c r="F53" s="24" t="n">
-        <v>46.03415337449829</v>
-      </c>
-      <c r="G53" s="24" t="n">
-        <v>78.73172057294317</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="n"/>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>vida_media_dias</t>
-        </is>
-      </c>
-      <c r="E54" s="24" t="n">
-        <v>27.83443881563776</v>
-      </c>
-      <c r="F54" s="24" t="n">
-        <v>43.34097095526067</v>
-      </c>
-      <c r="G54" s="24" t="n">
-        <v>87.6762263790841</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>vida_media_dias</t>
-        </is>
-      </c>
-      <c r="E55" s="24" t="n">
-        <v>69.85366986045834</v>
-      </c>
-      <c r="F55" s="24" t="n">
-        <v>6931.125226125684</v>
-      </c>
-      <c r="G55" s="24" t="n">
-        <v>6931.125226218031</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B56" s="4" t="n"/>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>vida_media_dias</t>
-        </is>
-      </c>
-      <c r="E56" s="24" t="n">
-        <v>43.50894829102631</v>
-      </c>
-      <c r="F56" s="24" t="n">
-        <v>398.3488886663965</v>
-      </c>
-      <c r="G56" s="24" t="n">
-        <v>6931.125226074509</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="n"/>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>vol_largo_plazo_anual</t>
-        </is>
-      </c>
-      <c r="E57" s="24" t="n">
-        <v>0.08601639430167922</v>
-      </c>
-      <c r="F57" s="24" t="n">
-        <v>0.09666244575535782</v>
-      </c>
-      <c r="G57" s="24" t="n">
-        <v>0.1118725413158892</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="n"/>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>vol_largo_plazo_anual</t>
-        </is>
-      </c>
-      <c r="E58" s="24" t="n">
-        <v>0.06485304098177484</v>
-      </c>
-      <c r="F58" s="24" t="n">
-        <v>0.07387492737579771</v>
-      </c>
-      <c r="G58" s="24" t="n">
-        <v>0.08647880318128304</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="n"/>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>vol_largo_plazo_anual</t>
-        </is>
-      </c>
-      <c r="E59" s="24" t="n">
-        <v>0.04647636256467483</v>
-      </c>
-      <c r="F59" s="24" t="n">
-        <v>0.0534943488527789</v>
-      </c>
-      <c r="G59" s="24" t="n">
-        <v>0.06887681095794745</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="n"/>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="D60" s="4" t="inlineStr">
-        <is>
-          <t>vol_largo_plazo_anual</t>
-        </is>
-      </c>
-      <c r="E60" s="24" t="n">
-        <v>0.0406913987162384</v>
-      </c>
-      <c r="F60" s="24" t="n">
-        <v>0.2641349192399155</v>
-      </c>
-      <c r="G60" s="24" t="n">
-        <v>0.3833351467838463</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>GARCH (residuos filtrados)</t>
-        </is>
-      </c>
-      <c r="B61" s="4" t="n"/>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>vol_largo_plazo_anual</t>
-        </is>
-      </c>
-      <c r="E61" s="24" t="n">
-        <v>0.02334179411047317</v>
-      </c>
-      <c r="F61" s="24" t="n">
-        <v>0.05546714102534646</v>
-      </c>
-      <c r="G61" s="24" t="n">
-        <v>0.2775739985773444</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>Pensiones: bootstrap estacionario de la historia (bloques de 12 meses en promedio), reestimando el HMM y repitiendo el Monte Carlo (hombre, 2.000 escenarios por historia).</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>HMM: bootstrap paramétrico con estados alineados a los originales (asignación húngara).</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>GARCH: simulación histórica filtrada (residuos estandarizados remuestreados). Persistencia 0,9999 = tope de la restricción (volatilidad integrada, vida media no acotada).</t>
+          <t>Grilla evaluada en escenarios de entrenamiento; resultados reportados en escenarios de prueba independientes.</t>
         </is>
       </c>
     </row>
@@ -30589,6 +29363,1582 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Incertidumbre de parámetros: intervalos de confianza de 90% por bootstrap (percentiles 5–95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>bloque</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>regimen</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>fondo</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>metrica</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>p05</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>mediana</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Pensiones (historia remuestreada)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>prima_real_A_vs_E</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="n">
+        <v>-0.02033327831223074</v>
+      </c>
+      <c r="F4" s="24" t="n">
+        <v>0.03465617575860558</v>
+      </c>
+      <c r="G4" s="24" t="n">
+        <v>0.07218940162832164</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Pensiones (historia remuestreada)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>cv_vs_defecto_mediana</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="n">
+        <v>-0.1414839611704128</v>
+      </c>
+      <c r="F5" s="24" t="n">
+        <v>0.3976446313068648</v>
+      </c>
+      <c r="G5" s="24" t="n">
+        <v>1.19503782136728</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Pensiones (historia remuestreada)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>cv_vs_defecto_p5</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="n">
+        <v>-0.2811320009079319</v>
+      </c>
+      <c r="F6" s="24" t="n">
+        <v>0.07979349629326404</v>
+      </c>
+      <c r="G6" s="24" t="n">
+        <v>0.6815268945114384</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Pensiones (historia remuestreada)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>prob_cv_supera_defecto</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="n">
+        <v>0.22735</v>
+      </c>
+      <c r="F7" s="24" t="n">
+        <v>0.92075</v>
+      </c>
+      <c r="G7" s="24" t="n">
+        <v>0.999525</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Pensiones (historia remuestreada)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>reactivo_vs_defecto_mediana</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="n">
+        <v>-0.08690068468870106</v>
+      </c>
+      <c r="F8" s="24" t="n">
+        <v>-0.03463701503838251</v>
+      </c>
+      <c r="G8" s="24" t="n">
+        <v>0.08547595265559825</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Pensiones (historia remuestreada)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>mediana_defecto_uf</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="n">
+        <v>6.425983355851145</v>
+      </c>
+      <c r="F9" s="24" t="n">
+        <v>10.94096361298217</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <v>18.88060876426169</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>persistencia</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="n">
+        <v>0.89955905324987</v>
+      </c>
+      <c r="F10" s="24" t="n">
+        <v>0.9501451205084048</v>
+      </c>
+      <c r="G10" s="24" t="n">
+        <v>0.9784178788593505</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>persistencia</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="n">
+        <v>0.6474081362214877</v>
+      </c>
+      <c r="F11" s="24" t="n">
+        <v>0.9833498083623404</v>
+      </c>
+      <c r="G11" s="24" t="n">
+        <v>0.9999999999978014</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>persistencia</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="n">
+        <v>0.2660517766209279</v>
+      </c>
+      <c r="F12" s="24" t="n">
+        <v>0.583671287299481</v>
+      </c>
+      <c r="G12" s="24" t="n">
+        <v>0.7756626825602544</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>duracion_meses</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="n">
+        <v>9.957652483720244</v>
+      </c>
+      <c r="F13" s="24" t="n">
+        <v>20.05835072661364</v>
+      </c>
+      <c r="G13" s="24" t="n">
+        <v>46.33960453807429</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>duracion_meses</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="n">
+        <v>2.837891664061405</v>
+      </c>
+      <c r="F14" s="24" t="n">
+        <v>60.09146038435532</v>
+      </c>
+      <c r="G14" s="24" t="n">
+        <v>454864035038.6853</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>duracion_meses</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="n">
+        <v>1.362495000031719</v>
+      </c>
+      <c r="F15" s="24" t="n">
+        <v>2.401949922421466</v>
+      </c>
+      <c r="G15" s="24" t="n">
+        <v>4.45763134079152</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>prob_estacionaria</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="n">
+        <v>3.910517304810142e-10</v>
+      </c>
+      <c r="F16" s="24" t="n">
+        <v>0.4847451207069491</v>
+      </c>
+      <c r="G16" s="24" t="n">
+        <v>0.8871964979924858</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>prob_estacionaria</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="n">
+        <v>0.0322741205452757</v>
+      </c>
+      <c r="F17" s="24" t="n">
+        <v>0.4256052965692377</v>
+      </c>
+      <c r="G17" s="24" t="n">
+        <v>0.9999999995623813</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>prob_estacionaria</t>
+        </is>
+      </c>
+      <c r="E18" s="24" t="n">
+        <v>3.683308530043981e-11</v>
+      </c>
+      <c r="F18" s="24" t="n">
+        <v>0.06387070500183775</v>
+      </c>
+      <c r="G18" s="24" t="n">
+        <v>0.1363100918200183</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>vol_A</t>
+        </is>
+      </c>
+      <c r="E19" s="24" t="n">
+        <v>0.08072897392403221</v>
+      </c>
+      <c r="F19" s="24" t="n">
+        <v>0.09235118502937775</v>
+      </c>
+      <c r="G19" s="24" t="n">
+        <v>0.1032374440937383</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>vol_A</t>
+        </is>
+      </c>
+      <c r="E20" s="24" t="n">
+        <v>0.08364058419755244</v>
+      </c>
+      <c r="F20" s="24" t="n">
+        <v>0.09981075731458454</v>
+      </c>
+      <c r="G20" s="24" t="n">
+        <v>0.1162739099861504</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>vol_A</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="n">
+        <v>0.1564126355374283</v>
+      </c>
+      <c r="F21" s="24" t="n">
+        <v>0.2530674011517392</v>
+      </c>
+      <c r="G21" s="24" t="n">
+        <v>0.3329043933475438</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>vol_B</t>
+        </is>
+      </c>
+      <c r="E22" s="24" t="n">
+        <v>0.06005314301343295</v>
+      </c>
+      <c r="F22" s="24" t="n">
+        <v>0.06867665571737128</v>
+      </c>
+      <c r="G22" s="24" t="n">
+        <v>0.07771607927689948</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>vol_B</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="n">
+        <v>0.0687710602341676</v>
+      </c>
+      <c r="F23" s="24" t="n">
+        <v>0.08079676866842468</v>
+      </c>
+      <c r="G23" s="24" t="n">
+        <v>0.09261084260112568</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>vol_B</t>
+        </is>
+      </c>
+      <c r="E24" s="24" t="n">
+        <v>0.1154395579469629</v>
+      </c>
+      <c r="F24" s="24" t="n">
+        <v>0.1828913218922641</v>
+      </c>
+      <c r="G24" s="24" t="n">
+        <v>0.2428672856036235</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>vol_C</t>
+        </is>
+      </c>
+      <c r="E25" s="24" t="n">
+        <v>0.04326168969124074</v>
+      </c>
+      <c r="F25" s="24" t="n">
+        <v>0.04878185657965282</v>
+      </c>
+      <c r="G25" s="24" t="n">
+        <v>0.05514623373205125</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>vol_C</t>
+        </is>
+      </c>
+      <c r="E26" s="24" t="n">
+        <v>0.05935831197621191</v>
+      </c>
+      <c r="F26" s="24" t="n">
+        <v>0.07051952792886923</v>
+      </c>
+      <c r="G26" s="24" t="n">
+        <v>0.08185603289511963</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>vol_C</t>
+        </is>
+      </c>
+      <c r="E27" s="24" t="n">
+        <v>0.0783586503246361</v>
+      </c>
+      <c r="F27" s="24" t="n">
+        <v>0.1262760922522181</v>
+      </c>
+      <c r="G27" s="24" t="n">
+        <v>0.164751908648498</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>vol_D</t>
+        </is>
+      </c>
+      <c r="E28" s="24" t="n">
+        <v>0.02729406917385757</v>
+      </c>
+      <c r="F28" s="24" t="n">
+        <v>0.0313933118895233</v>
+      </c>
+      <c r="G28" s="24" t="n">
+        <v>0.0359455172190928</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="4" t="n"/>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>vol_D</t>
+        </is>
+      </c>
+      <c r="E29" s="24" t="n">
+        <v>0.05929960760715521</v>
+      </c>
+      <c r="F29" s="24" t="n">
+        <v>0.07988590968454415</v>
+      </c>
+      <c r="G29" s="24" t="n">
+        <v>0.09224665384603417</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" s="4" t="n"/>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>vol_D</t>
+        </is>
+      </c>
+      <c r="E30" s="24" t="n">
+        <v>0.06581503427343903</v>
+      </c>
+      <c r="F30" s="24" t="n">
+        <v>0.09200615930554423</v>
+      </c>
+      <c r="G30" s="24" t="n">
+        <v>0.1203053956782151</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="4" t="n"/>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>vol_E</t>
+        </is>
+      </c>
+      <c r="E31" s="24" t="n">
+        <v>0.02153802834504729</v>
+      </c>
+      <c r="F31" s="24" t="n">
+        <v>0.02444829465876444</v>
+      </c>
+      <c r="G31" s="24" t="n">
+        <v>0.02714313140970778</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" s="4" t="n"/>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>vol_E</t>
+        </is>
+      </c>
+      <c r="E32" s="24" t="n">
+        <v>0.05854130433802626</v>
+      </c>
+      <c r="F32" s="24" t="n">
+        <v>0.08849692842917048</v>
+      </c>
+      <c r="G32" s="24" t="n">
+        <v>0.1022842599529493</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" s="4" t="n"/>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>vol_E</t>
+        </is>
+      </c>
+      <c r="E33" s="24" t="n">
+        <v>0.04960653960172515</v>
+      </c>
+      <c r="F33" s="24" t="n">
+        <v>0.07487598553830438</v>
+      </c>
+      <c r="G33" s="24" t="n">
+        <v>0.09562749248288493</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="4" t="n"/>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>pct_meses_reg1_desde_quiebre</t>
+        </is>
+      </c>
+      <c r="E34" s="24" t="n">
+        <v>0.2823863636363637</v>
+      </c>
+      <c r="F34" s="24" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="G34" s="24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="4" t="n"/>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>pct_meses_reg1_desde_quiebre</t>
+        </is>
+      </c>
+      <c r="E35" s="24" t="n">
+        <v>0.2823863636363637</v>
+      </c>
+      <c r="F35" s="24" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="G35" s="24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>HMM (paramétrico)</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" s="4" t="n"/>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>pct_meses_reg1_desde_quiebre</t>
+        </is>
+      </c>
+      <c r="E36" s="24" t="n">
+        <v>0.2823863636363637</v>
+      </c>
+      <c r="F36" s="24" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="G36" s="24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E37" s="24" t="n">
+        <v>0.07144614325844531</v>
+      </c>
+      <c r="F37" s="24" t="n">
+        <v>0.08754058087794941</v>
+      </c>
+      <c r="G37" s="24" t="n">
+        <v>0.1047518854535187</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n"/>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E38" s="24" t="n">
+        <v>0.07088467206040881</v>
+      </c>
+      <c r="F38" s="24" t="n">
+        <v>0.08319216147796728</v>
+      </c>
+      <c r="G38" s="24" t="n">
+        <v>0.09794931987327024</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n"/>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E39" s="24" t="n">
+        <v>0.07743559641469437</v>
+      </c>
+      <c r="F39" s="24" t="n">
+        <v>0.09323644048369883</v>
+      </c>
+      <c r="G39" s="24" t="n">
+        <v>0.1064908875409975</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n"/>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E40" s="24" t="n">
+        <v>0.1014273304397348</v>
+      </c>
+      <c r="F40" s="24" t="n">
+        <v>0.1229886920436335</v>
+      </c>
+      <c r="G40" s="24" t="n">
+        <v>0.1458810224153635</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="n"/>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="E41" s="24" t="n">
+        <v>0.08009149425301412</v>
+      </c>
+      <c r="F41" s="24" t="n">
+        <v>0.0962849069734741</v>
+      </c>
+      <c r="G41" s="24" t="n">
+        <v>0.1147972241326145</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="n"/>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="E42" s="24" t="n">
+        <v>0.870869662087573</v>
+      </c>
+      <c r="F42" s="24" t="n">
+        <v>0.8901119225657519</v>
+      </c>
+      <c r="G42" s="24" t="n">
+        <v>0.9087228392715047</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="n"/>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="E43" s="24" t="n">
+        <v>0.8847315189449467</v>
+      </c>
+      <c r="F43" s="24" t="n">
+        <v>0.9005922259810597</v>
+      </c>
+      <c r="G43" s="24" t="n">
+        <v>0.9158012795043712</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="n"/>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="E44" s="24" t="n">
+        <v>0.8732655999838247</v>
+      </c>
+      <c r="F44" s="24" t="n">
+        <v>0.8916758752359082</v>
+      </c>
+      <c r="G44" s="24" t="n">
+        <v>0.9107327299916633</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="E45" s="24" t="n">
+        <v>0.8540189775846361</v>
+      </c>
+      <c r="F45" s="24" t="n">
+        <v>0.8744521527367413</v>
+      </c>
+      <c r="G45" s="24" t="n">
+        <v>0.8905375360706199</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="n"/>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="E46" s="24" t="n">
+        <v>0.8808514806269054</v>
+      </c>
+      <c r="F46" s="24" t="n">
+        <v>0.9015989580759767</v>
+      </c>
+      <c r="G46" s="24" t="n">
+        <v>0.9149080365003966</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>persistencia</t>
+        </is>
+      </c>
+      <c r="E47" s="24" t="n">
+        <v>0.9670784595380398</v>
+      </c>
+      <c r="F47" s="24" t="n">
+        <v>0.9792250356075567</v>
+      </c>
+      <c r="G47" s="24" t="n">
+        <v>0.9868330247899996</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="n"/>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>persistencia</t>
+        </is>
+      </c>
+      <c r="E48" s="24" t="n">
+        <v>0.9762799801440459</v>
+      </c>
+      <c r="F48" s="24" t="n">
+        <v>0.9850554519333534</v>
+      </c>
+      <c r="G48" s="24" t="n">
+        <v>0.9912263501073139</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="n"/>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>persistencia</t>
+        </is>
+      </c>
+      <c r="E49" s="24" t="n">
+        <v>0.9754048323534276</v>
+      </c>
+      <c r="F49" s="24" t="n">
+        <v>0.9841341292347877</v>
+      </c>
+      <c r="G49" s="24" t="n">
+        <v>0.9921234543191135</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="n"/>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>persistencia</t>
+        </is>
+      </c>
+      <c r="E50" s="24" t="n">
+        <v>0.9901176467880164</v>
+      </c>
+      <c r="F50" s="24" t="n">
+        <v>0.9998999999999985</v>
+      </c>
+      <c r="G50" s="24" t="n">
+        <v>0.9998999999999998</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="n"/>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>persistencia</t>
+        </is>
+      </c>
+      <c r="E51" s="24" t="n">
+        <v>0.9841933602805655</v>
+      </c>
+      <c r="F51" s="24" t="n">
+        <v>0.9982613817048831</v>
+      </c>
+      <c r="G51" s="24" t="n">
+        <v>0.9998999999999977</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="n"/>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>vida_media_dias</t>
+        </is>
+      </c>
+      <c r="E52" s="24" t="n">
+        <v>20.70605048140716</v>
+      </c>
+      <c r="F52" s="24" t="n">
+        <v>33.01688513161351</v>
+      </c>
+      <c r="G52" s="24" t="n">
+        <v>52.29661231461255</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>vida_media_dias</t>
+        </is>
+      </c>
+      <c r="E53" s="24" t="n">
+        <v>28.87553394898189</v>
+      </c>
+      <c r="F53" s="24" t="n">
+        <v>46.03415337449829</v>
+      </c>
+      <c r="G53" s="24" t="n">
+        <v>78.73172057294317</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="n"/>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>vida_media_dias</t>
+        </is>
+      </c>
+      <c r="E54" s="24" t="n">
+        <v>27.83443881563776</v>
+      </c>
+      <c r="F54" s="24" t="n">
+        <v>43.34097095526067</v>
+      </c>
+      <c r="G54" s="24" t="n">
+        <v>87.6762263790841</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="n"/>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>vida_media_dias</t>
+        </is>
+      </c>
+      <c r="E55" s="24" t="n">
+        <v>69.85366986045834</v>
+      </c>
+      <c r="F55" s="24" t="n">
+        <v>6931.125226125684</v>
+      </c>
+      <c r="G55" s="24" t="n">
+        <v>6931.125226218031</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="n"/>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>vida_media_dias</t>
+        </is>
+      </c>
+      <c r="E56" s="24" t="n">
+        <v>43.50894829102631</v>
+      </c>
+      <c r="F56" s="24" t="n">
+        <v>398.3488886663965</v>
+      </c>
+      <c r="G56" s="24" t="n">
+        <v>6931.125226074509</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="n"/>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>vol_largo_plazo_anual</t>
+        </is>
+      </c>
+      <c r="E57" s="24" t="n">
+        <v>0.08601639430167922</v>
+      </c>
+      <c r="F57" s="24" t="n">
+        <v>0.09666244575535782</v>
+      </c>
+      <c r="G57" s="24" t="n">
+        <v>0.1118725413158892</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="n"/>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>vol_largo_plazo_anual</t>
+        </is>
+      </c>
+      <c r="E58" s="24" t="n">
+        <v>0.06485304098177484</v>
+      </c>
+      <c r="F58" s="24" t="n">
+        <v>0.07387492737579771</v>
+      </c>
+      <c r="G58" s="24" t="n">
+        <v>0.08647880318128304</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="n"/>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>vol_largo_plazo_anual</t>
+        </is>
+      </c>
+      <c r="E59" s="24" t="n">
+        <v>0.04647636256467483</v>
+      </c>
+      <c r="F59" s="24" t="n">
+        <v>0.0534943488527789</v>
+      </c>
+      <c r="G59" s="24" t="n">
+        <v>0.06887681095794745</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="n"/>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>vol_largo_plazo_anual</t>
+        </is>
+      </c>
+      <c r="E60" s="24" t="n">
+        <v>0.0406913987162384</v>
+      </c>
+      <c r="F60" s="24" t="n">
+        <v>0.2641349192399155</v>
+      </c>
+      <c r="G60" s="24" t="n">
+        <v>0.3833351467838463</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>GARCH (residuos filtrados)</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="n"/>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>vol_largo_plazo_anual</t>
+        </is>
+      </c>
+      <c r="E61" s="24" t="n">
+        <v>0.02334179411047317</v>
+      </c>
+      <c r="F61" s="24" t="n">
+        <v>0.05546714102534646</v>
+      </c>
+      <c r="G61" s="24" t="n">
+        <v>0.2775739985773444</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Pensiones: bootstrap estacionario de la historia (bloques de 12 meses en promedio), reestimando el HMM y repitiendo el Monte Carlo (hombre, 2.000 escenarios por historia).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>HMM: bootstrap paramétrico con estados alineados a los originales (asignación húngara).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>GARCH: simulación histórica filtrada (residuos estandarizados remuestreados). Persistencia 0,9999 = tope de la restricción (volatilidad integrada, vida media no acotada).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Microsimulación poblacional: 20.000 personas, lagunas y brecha de género (Shapley)
- microsimulacion.py: cohorte sintética con ingreso lognormal y densidad Beta por sexo
  calibrados con la SP (2026), lagunas como rachas de empleo formal (Markov) y mercado
  común a toda la cohorte; cálculo vectorizado como producto de matrices (BLAS).
- Hallazgo 13: la PGU vuelve la pensión muy progresiva (TR total 91% en Q1 a 50% en Q5,
  hombres); en 56% de los casos de mujeres la PGU es más de la mitad de la pensión.
- Hallazgo 14: descomposición de Shapley de la brecha de género (36%): la edad de
  pensión es la principal causa (41%), por sobre la densidad (27%) y el ingreso (18%).
- Figuras 13 y 14, hojas Excel, sección "Población y género" en el tablero. 35 pruebas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/reporte_proyecto_afp.xlsx
+++ b/reports/reporte_proyecto_afp.xlsx
@@ -26,8 +26,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pension_total" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pension_por_ingreso" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glidepath_optimo" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incertidumbre" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poblacion_sexo" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poblacion_quintil" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brecha_genero" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incertidumbre" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -535,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -751,6 +754,36 @@
       <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Maximizando la utilidad CRRA de la pensión total (hombre, consenso 2026, escenarios de prueba), el mejor glidepath de la familia supera al oficial en solo +0,3% a +3,1% de pensión equivalente cierta (aversión γ de 2 a 5); el fondo por defecto de la ley queda -9% a -1% bajo el oficial. Con γ = 3, el óptimo llega al retiro con 70% en crecimiento si se cuenta la PGU y 40% sin ella (el oficial, 29%): la PGU actúa como un bono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>En la población real la pensión depende sobre todo del ingreso y de las lagunas: la PGU la vuelve muy progresiva.</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Microsimulación de 20 mil personas con ingreso y densidad calibrados con la SP (consenso 2026, fondo por defecto): tasa de reemplazo total mediana 63% en hombres y 49% en mujeres (solo con el 10%: 27% y 14%). Del quintil 1 al 5 la tasa total baja de 91% a 50% (hombres). La PGU es más de la mitad de la pensión en 56% de los casos de mujeres. El ciclo de vida sube la pensión total +3% en el quintil 1 y +9% en el 5: la PGU amortigua su efecto en los de menores ingresos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>La edad de pensión explica la mayor parte de la brecha de género, más que las lagunas o el sueldo.</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>La pensión total mediana de una mujer es 36% menor que la de un hombre. Descomposición de Shapley: densidad de cotización 9,7 pp; nivel de ingreso 6,6 pp; edad de pensión (60 vs 65) 14,8 pp; esperanza de vida (tabla de mortalidad) 4,1 pp. El factor más importante es «Edad de pensión (60 vs 65)», con 41% de la brecha.</t>
         </is>
       </c>
     </row>
@@ -29363,6 +29396,789 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Microsimulación poblacional: resultados por sexo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>sexo</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>personas</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>densidad_media</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>sueldo_ref_mediano_uf</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>pension_10_mediana</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>pension_total_mediana</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>tr_10_mediana</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>tr_total_mediana</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>prob_tr_meta_10</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>prob_tr_meta_total</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>pct_pgu_mayor_mitad</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>cv_vs_defecto_mediana</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>pct_personas_cv_gana</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>pct_sin_pension</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>11239</v>
+      </c>
+      <c r="C4" s="22" t="n">
+        <v>0.5805993638224041</v>
+      </c>
+      <c r="D4" s="25" t="n">
+        <v>26.25829840045317</v>
+      </c>
+      <c r="E4" s="25" t="n">
+        <v>7.481994497828804</v>
+      </c>
+      <c r="F4" s="25" t="n">
+        <v>17.38973362563933</v>
+      </c>
+      <c r="G4" s="22" t="n">
+        <v>0.2670172714202461</v>
+      </c>
+      <c r="H4" s="22" t="n">
+        <v>0.627175283115325</v>
+      </c>
+      <c r="I4" s="22" t="n">
+        <v>0.2357874366046801</v>
+      </c>
+      <c r="J4" s="22" t="n">
+        <v>0.8232382774268173</v>
+      </c>
+      <c r="K4" s="22" t="n">
+        <v>0.3241498353946081</v>
+      </c>
+      <c r="L4" s="22" t="n">
+        <v>0.05220831349824118</v>
+      </c>
+      <c r="M4" s="22" t="n">
+        <v>0.9652994038615536</v>
+      </c>
+      <c r="N4" s="22" t="n">
+        <v>0.001156686537948204</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>8761</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.4988751555867181</v>
+      </c>
+      <c r="D5" s="25" t="n">
+        <v>22.78885777217155</v>
+      </c>
+      <c r="E5" s="25" t="n">
+        <v>3.409478324138548</v>
+      </c>
+      <c r="F5" s="25" t="n">
+        <v>11.29128401947322</v>
+      </c>
+      <c r="G5" s="22" t="n">
+        <v>0.1448364045296125</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <v>0.4868260432354977</v>
+      </c>
+      <c r="I5" s="22" t="n">
+        <v>0.02233477913480196</v>
+      </c>
+      <c r="J5" s="22" t="n">
+        <v>0.6610569569683826</v>
+      </c>
+      <c r="K5" s="22" t="n">
+        <v>0.5577331354868166</v>
+      </c>
+      <c r="L5" s="22" t="n">
+        <v>0.04604804290898745</v>
+      </c>
+      <c r="M5" s="22" t="n">
+        <v>0.9344823650268235</v>
+      </c>
+      <c r="N5" s="22" t="n">
+        <v>0.001255564433283896</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Cohorte sintética que empieza a cotizar a los 25 en 2026. Ingreso lognormal y densidad Beta por sexo calibrados con la SP (2026);</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>lagunas como rachas de empleo formal (cadena de Markov); supuestos de mercado de consenso 2026; fondo por defecto salvo cv_*.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Métricas por persona: mediana sobre 400 escenarios de mercado comunes a toda la cohorte.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Microsimulación: tasa de reemplazo y PGU por quintil de ingreso</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>sexo</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>quintil</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>sueldo_ref_mediano_uf</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>tr_10_mediana</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>tr_total_mediana</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>prob_tr_meta_total</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>pgu_mediana</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>pension_total_mediana</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>cv_vs_defecto_total</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>cv_vs_defecto_propia</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="25" t="n">
+        <v>10.0890592393075</v>
+      </c>
+      <c r="D4" s="22" t="n">
+        <v>0.1970876041893812</v>
+      </c>
+      <c r="E4" s="22" t="n">
+        <v>0.9055514372578255</v>
+      </c>
+      <c r="F4" s="22" t="n">
+        <v>0.9988067170818505</v>
+      </c>
+      <c r="G4" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="H4" s="25" t="n">
+        <v>9.515179911634196</v>
+      </c>
+      <c r="I4" s="22" t="n">
+        <v>0.03225722708868506</v>
+      </c>
+      <c r="J4" s="22" t="n">
+        <v>0.09441231508530556</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="25" t="n">
+        <v>17.6492084296502</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>0.2372533021486117</v>
+      </c>
+      <c r="E5" s="22" t="n">
+        <v>0.669052509116302</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.8609219306049822</v>
+      </c>
+      <c r="G5" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="H5" s="25" t="n">
+        <v>13.57942737452789</v>
+      </c>
+      <c r="I5" s="22" t="n">
+        <v>0.05206309830474876</v>
+      </c>
+      <c r="J5" s="22" t="n">
+        <v>0.09143316457570294</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="25" t="n">
+        <v>26.25829840045317</v>
+      </c>
+      <c r="D6" s="22" t="n">
+        <v>0.2663475193457446</v>
+      </c>
+      <c r="E6" s="22" t="n">
+        <v>0.6102772824816237</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.7845649755229195</v>
+      </c>
+      <c r="G6" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="H6" s="25" t="n">
+        <v>18.51658087864134</v>
+      </c>
+      <c r="I6" s="22" t="n">
+        <v>0.05126404819025376</v>
+      </c>
+      <c r="J6" s="22" t="n">
+        <v>0.09171624295446779</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="25" t="n">
+        <v>39.03507537049039</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>0.2885022240977092</v>
+      </c>
+      <c r="E7" s="22" t="n">
+        <v>0.5525413219485328</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>0.7541270017793594</v>
+      </c>
+      <c r="G7" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="H7" s="25" t="n">
+        <v>26.05048364586172</v>
+      </c>
+      <c r="I7" s="22" t="n">
+        <v>0.05322642747730222</v>
+      </c>
+      <c r="J7" s="22" t="n">
+        <v>0.09062953534217799</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <v>67.73478483449657</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>0.3304236211681073</v>
+      </c>
+      <c r="E8" s="22" t="n">
+        <v>0.5027594985976973</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>0.7177535587188613</v>
+      </c>
+      <c r="G8" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="25" t="n">
+        <v>37.79947549952672</v>
+      </c>
+      <c r="I8" s="22" t="n">
+        <v>0.09139904408910704</v>
+      </c>
+      <c r="J8" s="22" t="n">
+        <v>0.08930687859248865</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="25" t="n">
+        <v>8.220943761205294</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>0.1000789667757265</v>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>0.8749511718502516</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="H9" s="25" t="n">
+        <v>7.62278818472261</v>
+      </c>
+      <c r="I9" s="22" t="n">
+        <v>0.01836549528759068</v>
+      </c>
+      <c r="J9" s="22" t="n">
+        <v>0.1225891130383312</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="25" t="n">
+        <v>15.06507534093625</v>
+      </c>
+      <c r="D10" s="22" t="n">
+        <v>0.1278117279541412</v>
+      </c>
+      <c r="E10" s="22" t="n">
+        <v>0.5573505770314425</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>0.8540924657534247</v>
+      </c>
+      <c r="G10" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="H10" s="25" t="n">
+        <v>9.625103119302095</v>
+      </c>
+      <c r="I10" s="22" t="n">
+        <v>0.03725086236125719</v>
+      </c>
+      <c r="J10" s="22" t="n">
+        <v>0.1182546318284345</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>22.789244250418</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>0.1430008860534954</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <v>0.4546856376626829</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>0.6190139840182648</v>
+      </c>
+      <c r="G11" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="H11" s="25" t="n">
+        <v>11.98320641609059</v>
+      </c>
+      <c r="I11" s="22" t="n">
+        <v>0.05013557461240958</v>
+      </c>
+      <c r="J11" s="22" t="n">
+        <v>0.1040122345109671</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>34.48010670630391</v>
+      </c>
+      <c r="D12" s="22" t="n">
+        <v>0.159219029977004</v>
+      </c>
+      <c r="E12" s="22" t="n">
+        <v>0.3968568078220203</v>
+      </c>
+      <c r="F12" s="22" t="n">
+        <v>0.4924429223744292</v>
+      </c>
+      <c r="G12" s="25" t="n">
+        <v>6.303600438248517</v>
+      </c>
+      <c r="H12" s="25" t="n">
+        <v>15.91498209493261</v>
+      </c>
+      <c r="I12" s="22" t="n">
+        <v>0.0547507385456214</v>
+      </c>
+      <c r="J12" s="22" t="n">
+        <v>0.1177811378312603</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="25" t="n">
+        <v>62.82966770704746</v>
+      </c>
+      <c r="D13" s="22" t="n">
+        <v>0.1883770187870422</v>
+      </c>
+      <c r="E13" s="22" t="n">
+        <v>0.338229335071116</v>
+      </c>
+      <c r="F13" s="22" t="n">
+        <v>0.3395419520547945</v>
+      </c>
+      <c r="G13" s="25" t="n">
+        <v>0.4497467459310651</v>
+      </c>
+      <c r="H13" s="25" t="n">
+        <v>24.07750780202309</v>
+      </c>
+      <c r="I13" s="22" t="n">
+        <v>0.06879387571046225</v>
+      </c>
+      <c r="J13" s="22" t="n">
+        <v>0.1180706210236555</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Cohorte sintética que empieza a cotizar a los 25 en 2026. Ingreso lognormal y densidad Beta por sexo calibrados con la SP (2026);</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>lagunas como rachas de empleo formal (cadena de Markov); supuestos de mercado de consenso 2026; fondo por defecto salvo cv_*.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Métricas por persona: mediana sobre 400 escenarios de mercado comunes a toda la cohorte.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Descomposición de Shapley de la brecha de pensión total mediana mujer/hombre</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>factor</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>aporte_uf</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>aporte_pp_brecha</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Densidad de cotización</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="n">
+        <v>1.720811102106209</v>
+      </c>
+      <c r="C4" s="22" t="n">
+        <v>0.09740884310220008</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Nivel de ingreso</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="n">
+        <v>1.163122203027938</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.065840107635731</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Edad de pensión (60 vs 65)</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="n">
+        <v>2.612171037987555</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.1478654795311381</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Esperanza de vida (tabla de mortalidad)</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="n">
+        <v>0.7289185736611913</v>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>0.0412614231097982</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Residuo (fondo por defecto por sexo y muestreo)</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="n">
+        <v>0.1177015996468711</v>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>0.006662658463120724</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Aporte = efecto marginal promedio de asignar a las mujeres la característica de los hombres, sobre todos los órdenes.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -30933,7 +31749,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Regímenes con variables macro (TVTP-HMM) y licencias MIT / CC BY 4.0
- scripts/descarga_mindicador.py: IPC, TPM, dólar e Imacec desde la API pública de
  mindicador.cl (sin credenciales), rezagados según su calendario de publicación.
- regimenes_macro.py: HMM con probabilidades de transición variables (EM propio,
  regresión logística multinomial ponderada con ridge), evaluación walk-forward
  2015-2026 con densidad predictiva a un paso y test de Diebold-Mariano HAC.
- Hallazgo 15: los regímenes predicen mejor que una normal (p < 0,001), pero la macro
  no agrega capacidad predictiva fuera de muestra (p = 0,98), con cualquier ridge.
- Figura 15, hojas Excel, documento de trabajo actualizado. 39 pruebas.
- LICENSE (MIT, código) y LICENSE-CONTENIDO.md (CC BY 4.0, documentos y figuras).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/reporte_proyecto_afp.xlsx
+++ b/reports/reporte_proyecto_afp.xlsx
@@ -26,11 +26,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pension_total" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pension_por_ingreso" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glidepath_optimo" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poblacion_sexo" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poblacion_quintil" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brecha_genero" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incertidumbre" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regimenes_macro" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regimenes_macro_efectos" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poblacion_sexo" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poblacion_quintil" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brecha_genero" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incertidumbre" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,12 +41,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="$#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="#,##0.0"/>
+    <numFmt numFmtId="169" formatCode="0.000"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -137,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -173,6 +176,7 @@
     <xf numFmtId="168" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -538,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -778,12 +782,27 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>La edad de pensión explica la mayor parte de la brecha de género, más que las lagunas o el sueldo.</t>
+          <t>La edad de pensión es la principal causa de la brecha de género, por sobre las lagunas y el sueldo.</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
           <t>La pensión total mediana de una mujer es 36% menor que la de un hombre. Descomposición de Shapley: densidad de cotización 9,7 pp; nivel de ingreso 6,6 pp; edad de pensión (60 vs 65) 14,8 pp; esperanza de vida (tabla de mortalidad) 4,1 pp. El factor más importante es «Edad de pensión (60 vs 65)», con 41% de la brecha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Los regímenes mejoran la predicción del mes siguiente, pero las variables macro no ayudan a anticiparlos.</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Validación fuera de muestra 2015-2026 (140 meses, reestimación anual): el HMM supera a una normal sin regímenes en +0,74 de log-score por mes (Diebold-Mariano p = 0,001). Agregar IPC, TPM, dólar e Imacec a las transiciones (TVTP) no mejora: -0,001 por mes (p = 0,98). Dentro de muestra, una TPM que sube 1 desviación estándar eleva la probabilidad de pasar de la calma a la crisis de 4% a 16%, pero el quiebre de 2019 ocurrió una sola vez: no hay transiciones suficientes para aprender qué lo gatilla.</t>
         </is>
       </c>
     </row>
@@ -29396,6 +29415,750 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>¿Ayuda la macro a predecir? Densidad predictiva a un paso fuera de muestra (walk-forward 2015-2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>log_score_promedio</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>meses</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>tvtp_menos_modelo</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>t_diebold_mariano</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>p_valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>HMM constante</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="n">
+        <v>18.19688060959884</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>140</v>
+      </c>
+      <c r="D4" s="24" t="n">
+        <v>-0.0007646710963605142</v>
+      </c>
+      <c r="E4" s="25" t="n">
+        <v>-0.02068102037143527</v>
+      </c>
+      <c r="F4" s="29" t="n">
+        <v>0.983500109332232</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>HMM con macro (TVTP)</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="n">
+        <v>18.19611593850247</v>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>140</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="25" t="n">
+        <v/>
+      </c>
+      <c r="F5" s="29" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Normal (sin regímenes)</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>17.45985243974132</v>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>140</v>
+      </c>
+      <c r="D6" s="24" t="n">
+        <v>0.7362634987611505</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>3.412504525197265</v>
+      </c>
+      <c r="F6" s="29" t="n">
+        <v>0.0006436885824909755</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Log-score = log p(retornos del mes siguiente | información hasta hoy); mayor es mejor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Diebold-Mariano con varianza HAC (Newey-West, 6 rezagos) sobre la diferencia mensual TVTP − modelo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TVTP: probabilidades de transición = softmax(b + w·z), z = inflación 12m, ΔTPM 6m, dólar 3m, Imacec (rezagados).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Efecto de +1 desviación estándar de cada variable sobre la probabilidad de cambiar de régimen (muestra completa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>variable</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>desde</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>hacia</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>prob_base</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>prob_con_+1sd</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>cambio_pp</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Inflación 12 meses (IPC, rezago 1 mes)</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="22" t="n">
+        <v>0.007113533538454774</v>
+      </c>
+      <c r="E4" s="22" t="n">
+        <v>0.006147412547967908</v>
+      </c>
+      <c r="F4" s="22" t="n">
+        <v>-0.0009661209904868661</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Inflación 12 meses (IPC, rezago 1 mes)</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>0.04027952998959874</v>
+      </c>
+      <c r="E5" s="22" t="n">
+        <v>0.1083892813005483</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.06810975131094954</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Inflación 12 meses (IPC, rezago 1 mes)</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="22" t="n">
+        <v>3.626380783916921e-07</v>
+      </c>
+      <c r="E6" s="22" t="n">
+        <v>3.647593157782228e-07</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>2.121237386530683e-09</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Inflación 12 meses (IPC, rezago 1 mes)</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>0.01386195391553562</v>
+      </c>
+      <c r="E7" s="22" t="n">
+        <v>0.008074657056739118</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>-0.0057872968587965</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Inflación 12 meses (IPC, rezago 1 mes)</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>0.4727230182583151</v>
+      </c>
+      <c r="E8" s="22" t="n">
+        <v>0.4589743682034549</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>-0.01374865005486015</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Inflación 12 meses (IPC, rezago 1 mes)</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>3.67627007744074e-06</v>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>3.771968725577081e-06</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>9.569864813634134e-08</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Cambio de la TPM en 6 meses</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="22" t="n">
+        <v>0.007113533538454774</v>
+      </c>
+      <c r="E10" s="22" t="n">
+        <v>0.008211044641741046</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>0.001097511103286273</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Cambio de la TPM en 6 meses</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>0.04027952998959874</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <v>0.1641658946386991</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>0.1238863646491004</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Cambio de la TPM en 6 meses</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="22" t="n">
+        <v>3.626380783916921e-07</v>
+      </c>
+      <c r="E12" s="22" t="n">
+        <v>3.64110863939917e-07</v>
+      </c>
+      <c r="F12" s="22" t="n">
+        <v>1.47278554822494e-09</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Cambio de la TPM en 6 meses</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="22" t="n">
+        <v>0.01386195391553562</v>
+      </c>
+      <c r="E13" s="22" t="n">
+        <v>0.009851759947025642</v>
+      </c>
+      <c r="F13" s="22" t="n">
+        <v>-0.004010193968509976</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Cambio de la TPM en 6 meses</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="22" t="n">
+        <v>0.4727230182583151</v>
+      </c>
+      <c r="E14" s="22" t="n">
+        <v>0.5065065435534337</v>
+      </c>
+      <c r="F14" s="22" t="n">
+        <v>0.03378352529511863</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Cambio de la TPM en 6 meses</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="22" t="n">
+        <v>3.67627007744074e-06</v>
+      </c>
+      <c r="E15" s="22" t="n">
+        <v>3.440886989554388e-06</v>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>-2.353830878863523e-07</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Variación del dólar en 3 meses</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="22" t="n">
+        <v>0.007113533538454774</v>
+      </c>
+      <c r="E16" s="22" t="n">
+        <v>0.006223658201725711</v>
+      </c>
+      <c r="F16" s="22" t="n">
+        <v>-0.0008898753367290631</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Variación del dólar en 3 meses</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="22" t="n">
+        <v>0.04027952998959874</v>
+      </c>
+      <c r="E17" s="22" t="n">
+        <v>0.03101232277030021</v>
+      </c>
+      <c r="F17" s="22" t="n">
+        <v>-0.00926720721929853</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Variación del dólar en 3 meses</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="22" t="n">
+        <v>3.626380783916921e-07</v>
+      </c>
+      <c r="E18" s="22" t="n">
+        <v>3.613501175739493e-07</v>
+      </c>
+      <c r="F18" s="22" t="n">
+        <v>-1.287960817742857e-09</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Variación del dólar en 3 meses</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="22" t="n">
+        <v>0.01386195391553562</v>
+      </c>
+      <c r="E19" s="22" t="n">
+        <v>0.01736274185592507</v>
+      </c>
+      <c r="F19" s="22" t="n">
+        <v>0.003500787940389454</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Variación del dólar en 3 meses</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="22" t="n">
+        <v>0.4727230182583151</v>
+      </c>
+      <c r="E20" s="22" t="n">
+        <v>0.45913699666999</v>
+      </c>
+      <c r="F20" s="22" t="n">
+        <v>-0.01358602158832511</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Variación del dólar en 3 meses</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="22" t="n">
+        <v>3.67627007744074e-06</v>
+      </c>
+      <c r="E21" s="22" t="n">
+        <v>3.770954715106118e-06</v>
+      </c>
+      <c r="F21" s="22" t="n">
+        <v>9.468463766537803e-08</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Imacec anual (rezago 2 meses)</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="22" t="n">
+        <v>0.007113533538454774</v>
+      </c>
+      <c r="E22" s="22" t="n">
+        <v>0.002220170341564814</v>
+      </c>
+      <c r="F22" s="22" t="n">
+        <v>-0.00489336319688996</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Imacec anual (rezago 2 meses)</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="22" t="n">
+        <v>0.04027952998959874</v>
+      </c>
+      <c r="E23" s="22" t="n">
+        <v>0.02939155221399957</v>
+      </c>
+      <c r="F23" s="22" t="n">
+        <v>-0.01088797777559918</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Imacec anual (rezago 2 meses)</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="22" t="n">
+        <v>3.626380783916921e-07</v>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>3.619939466047499e-07</v>
+      </c>
+      <c r="F24" s="22" t="n">
+        <v>-6.441317869422473e-10</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Imacec anual (rezago 2 meses)</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="22" t="n">
+        <v>0.01386195391553562</v>
+      </c>
+      <c r="E25" s="22" t="n">
+        <v>0.01561265704507581</v>
+      </c>
+      <c r="F25" s="22" t="n">
+        <v>0.001750703129540192</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Imacec anual (rezago 2 meses)</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="22" t="n">
+        <v>0.4727230182583151</v>
+      </c>
+      <c r="E26" s="22" t="n">
+        <v>0.5334271889808903</v>
+      </c>
+      <c r="F26" s="22" t="n">
+        <v>0.06070417072257517</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Imacec anual (rezago 2 meses)</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="22" t="n">
+        <v>3.67627007744074e-06</v>
+      </c>
+      <c r="E27" s="22" t="n">
+        <v>3.253062541141058e-06</v>
+      </c>
+      <c r="F27" s="22" t="n">
+        <v>-4.232075362996822e-07</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Regímenes: 0 = calma, 1 = tasas volátiles (post-2019), 2 = crisis bursátil.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -29612,7 +30375,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -30058,7 +30821,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -30173,7 +30936,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31749,13 +32512,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -31835,6 +32598,13 @@
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Reforma de pensiones: Ley N.º 21.735; Subsecretaría de Previsión Social, Nota Técnica (ago-2025), tablas 1, 3 y 5. PGU y umbrales de pensión base: SP (vigentes desde el 01-02-2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Variables macro (IPC, TPM, dólar observado, Imacec): API pública de mindicador.cl, que republica series del BCCh y el INE.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Comisiones por AFP: costo en pensión y rentabilidad necesaria para compensarlo
- comisiones.py: costo de la comisión expresado en pensión (lineal en aportes), punto
  de equilibrio de rentabilidad por bisección sobre escenarios de consenso, y
  rentabilidad relativa de cada AFP frente a sus pares con su error estándar.
- Hallazgo 16: la AFP más cara equivale a perder 9,9% de la pensión autofinanciada;
  ninguna AFP rindió lo suficiente para compensar su comisión (nov-2019 a ago-2026).
- Figura 16, hoja Excel Comisiones_AFP, sección en el tablero, documento de trabajo
  (4.7 y nueva implicancia de política). 41 pruebas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/reporte_proyecto_afp.xlsx
+++ b/reports/reporte_proyecto_afp.xlsx
@@ -26,13 +26,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pension_total" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pension_por_ingreso" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glidepath_optimo" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regimenes_macro" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regimenes_macro_efectos" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poblacion_sexo" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poblacion_quintil" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brecha_genero" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incertidumbre" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comisiones_AFP" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regimenes_macro" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regimenes_macro_efectos" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poblacion_sexo" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poblacion_quintil" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brecha_genero" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incertidumbre" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -140,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -176,6 +177,7 @@
     <xf numFmtId="168" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -542,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -797,10 +799,25 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
+          <t>Pagar más comisión no compra más rentabilidad: ninguna AFP rindió lo suficiente para compensar su comisión.</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Las comisiones van de 0,46% (Uno) a 1,45% (Provida) del sueldo. Como se cobran aparte de la cotización, la diferencia equivale a dejar de ahorrar 9,9% de la pensión autofinanciada (0,96 UF al mes para el hombre tipo; 135 vs 43 UF pagadas en la vida laboral). Para compensarla, Provida necesitaría rendir 0,41% más al año; entre nov-2019 y ago-2026 rindió -0,16% frente a sus pares (t vs equilibrio -2,1). La que más rindió (Capital, +0,25%) tampoco alcanzó su equilibrio (0,41%), y ninguna diferencia de rentabilidad es significativa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
           <t>Los regímenes mejoran la predicción del mes siguiente, pero las variables macro no ayudan a anticiparlos.</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Validación fuera de muestra 2015-2026 (140 meses, reestimación anual): el HMM supera a una normal sin regímenes en +0,74 de log-score por mes (Diebold-Mariano p = 0,001). Agregar IPC, TPM, dólar e Imacec a las transiciones (TVTP) no mejora: -0,001 por mes (p = 0,98). Dentro de muestra, una TPM que sube 1 desviación estándar eleva la probabilidad de pasar de la calma a la crisis de 4% a 16%, pero el quiebre de 2019 ocurrió una sola vez: no hay transiciones suficientes para aprender qué lo gatilla.</t>
         </is>
@@ -29415,6 +29432,492 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Comisiones por AFP: costo en pensión y rentabilidad necesaria para compensarlo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>afp</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>comision</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>comision_mensual_clp_sueldo_1m</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>comision_total_vida_uf</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>costo_pension_uf_vs_mas_barata</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>costo_pension_pct_vs_mas_barata</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>rentabilidad_extra_para_compensar</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>alfa_historico</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>meses_historico</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>ee_alfa_historico</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>alfa_comun</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>meses_comun</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>ee_alfa_comun</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>alfa_menos_equilibrio</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>t_vs_equilibrio</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Uno</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="C4" s="29" t="n">
+        <v>4600</v>
+      </c>
+      <c r="D4" s="23" t="n">
+        <v>42.91292484478021</v>
+      </c>
+      <c r="E4" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="22" t="n">
+        <v>0.002357478638588062</v>
+      </c>
+      <c r="I4" s="14" t="n">
+        <v>83</v>
+      </c>
+      <c r="J4" s="22" t="n">
+        <v>0.004551510994692204</v>
+      </c>
+      <c r="K4" s="22" t="n">
+        <v>-0.0002357973628636101</v>
+      </c>
+      <c r="L4" s="14" t="n">
+        <v>82</v>
+      </c>
+      <c r="M4" s="22" t="n">
+        <v>0.003618040065530605</v>
+      </c>
+      <c r="N4" s="22" t="n">
+        <v>-0.0002357973628636101</v>
+      </c>
+      <c r="O4" s="25" t="n">
+        <v>-0.06517267874119828</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="n">
+        <v>0.0058</v>
+      </c>
+      <c r="C5" s="29" t="n">
+        <v>5800</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>54.10760089124459</v>
+      </c>
+      <c r="E5" s="25" t="n">
+        <v>0.1168610627846689</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="G5" s="22" t="n">
+        <v>0.0005168151855468751</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <v>-0.001346627810657086</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>192</v>
+      </c>
+      <c r="J5" s="22" t="n">
+        <v>0.002267516752812703</v>
+      </c>
+      <c r="K5" s="22" t="n">
+        <v>-0.002230214467713254</v>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>82</v>
+      </c>
+      <c r="M5" s="22" t="n">
+        <v>0.002529811826278836</v>
+      </c>
+      <c r="N5" s="22" t="n">
+        <v>-0.002747029653260129</v>
+      </c>
+      <c r="O5" s="25" t="n">
+        <v>-1.085863234856011</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>PlanVital</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="n">
+        <v>0.0116</v>
+      </c>
+      <c r="C6" s="29" t="n">
+        <v>11600</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>108.2152017824892</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>0.6816895329105687</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.06999999999999999</v>
+      </c>
+      <c r="G6" s="22" t="n">
+        <v>0.002936553955078125</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <v>-0.001648877451749176</v>
+      </c>
+      <c r="I6" s="14" t="n">
+        <v>289</v>
+      </c>
+      <c r="J6" s="22" t="n">
+        <v>0.001587436154611429</v>
+      </c>
+      <c r="K6" s="22" t="n">
+        <v>0.000927368629194536</v>
+      </c>
+      <c r="L6" s="14" t="n">
+        <v>82</v>
+      </c>
+      <c r="M6" s="22" t="n">
+        <v>0.002153718936999545</v>
+      </c>
+      <c r="N6" s="22" t="n">
+        <v>-0.002009185325883589</v>
+      </c>
+      <c r="O6" s="25" t="n">
+        <v>-0.932891145342617</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Habitat</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="n">
+        <v>0.0127</v>
+      </c>
+      <c r="C7" s="29" t="n">
+        <v>12700</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>118.476988158415</v>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>0.7888121737965151</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>0.08099999999999999</v>
+      </c>
+      <c r="G7" s="22" t="n">
+        <v>0.003376922607421875</v>
+      </c>
+      <c r="H7" s="22" t="n">
+        <v>0.003300291758884022</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>289</v>
+      </c>
+      <c r="J7" s="22" t="n">
+        <v>0.001180359962717409</v>
+      </c>
+      <c r="K7" s="22" t="n">
+        <v>0.00137962531723097</v>
+      </c>
+      <c r="L7" s="14" t="n">
+        <v>82</v>
+      </c>
+      <c r="M7" s="22" t="n">
+        <v>0.002208891381672083</v>
+      </c>
+      <c r="N7" s="22" t="n">
+        <v>-0.001997297290190905</v>
+      </c>
+      <c r="O7" s="25" t="n">
+        <v>-0.904208014374611</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Capital</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="n">
+        <v>0.0144</v>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>14400</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>134.3361125575728</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>0.9543653460747962</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>0.09799999999999999</v>
+      </c>
+      <c r="G8" s="22" t="n">
+        <v>0.004052581787109375</v>
+      </c>
+      <c r="H8" s="22" t="n">
+        <v>0.001075497427890193</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>221</v>
+      </c>
+      <c r="J8" s="22" t="n">
+        <v>0.001161323746836198</v>
+      </c>
+      <c r="K8" s="22" t="n">
+        <v>0.002530410792174975</v>
+      </c>
+      <c r="L8" s="14" t="n">
+        <v>82</v>
+      </c>
+      <c r="M8" s="22" t="n">
+        <v>0.001474062914294543</v>
+      </c>
+      <c r="N8" s="22" t="n">
+        <v>-0.0015221709949344</v>
+      </c>
+      <c r="O8" s="25" t="n">
+        <v>-1.032636382187853</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Cuprum</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="n">
+        <v>0.0144</v>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>14400</v>
+      </c>
+      <c r="D9" s="23" t="n">
+        <v>134.3361125575728</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>0.9543653460747962</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>0.09799999999999999</v>
+      </c>
+      <c r="G9" s="22" t="n">
+        <v>0.004052581787109375</v>
+      </c>
+      <c r="H9" s="22" t="n">
+        <v>0.001529268021796026</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>289</v>
+      </c>
+      <c r="J9" s="22" t="n">
+        <v>0.001294373993724194</v>
+      </c>
+      <c r="K9" s="22" t="n">
+        <v>0.001324839680963974</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>82</v>
+      </c>
+      <c r="M9" s="22" t="n">
+        <v>0.001911337442733075</v>
+      </c>
+      <c r="N9" s="22" t="n">
+        <v>-0.002727742106145402</v>
+      </c>
+      <c r="O9" s="25" t="n">
+        <v>-1.427137901010785</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Provida</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="n">
+        <v>0.0145</v>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>14500</v>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>135.2690022281115</v>
+      </c>
+      <c r="E10" s="25" t="n">
+        <v>0.9641037679735187</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="G10" s="22" t="n">
+        <v>0.004091949462890626</v>
+      </c>
+      <c r="H10" s="22" t="n">
+        <v>-0.002006289828630292</v>
+      </c>
+      <c r="I10" s="14" t="n">
+        <v>289</v>
+      </c>
+      <c r="J10" s="22" t="n">
+        <v>0.001258910262090376</v>
+      </c>
+      <c r="K10" s="22" t="n">
+        <v>-0.001569775613138447</v>
+      </c>
+      <c r="L10" s="14" t="n">
+        <v>82</v>
+      </c>
+      <c r="M10" s="22" t="n">
+        <v>0.002646277164591531</v>
+      </c>
+      <c r="N10" s="22" t="n">
+        <v>-0.005661725076029073</v>
+      </c>
+      <c r="O10" s="25" t="n">
+        <v>-2.139505699473091</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Comisión = % del sueldo imponible, aparte del 10% (SP, vigente desde el 01-10-2025).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Costo en pensión = (comisión − comisión más baja) / 10% × pensión autofinanciada (la pensión es lineal en los aportes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Rentabilidad extra para compensar = retorno real anual adicional que iguala esa pensión (fondo por defecto, consenso 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Alfa = rentabilidad real anual frente al promedio ponderado de las demás AFP, promedio de los 5 fondos; común = nov-2019 a ago-2026 (las 7 AFP). t_vs_equilibrio = (alfa − necesaria) / error estándar.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -29483,7 +29986,7 @@
       <c r="E4" s="25" t="n">
         <v>-0.02068102037143527</v>
       </c>
-      <c r="F4" s="29" t="n">
+      <c r="F4" s="30" t="n">
         <v>0.983500109332232</v>
       </c>
     </row>
@@ -29505,7 +30008,7 @@
       <c r="E5" s="25" t="n">
         <v/>
       </c>
-      <c r="F5" s="29" t="n">
+      <c r="F5" s="30" t="n">
         <v/>
       </c>
     </row>
@@ -29527,7 +30030,7 @@
       <c r="E6" s="25" t="n">
         <v>3.412504525197265</v>
       </c>
-      <c r="F6" s="29" t="n">
+      <c r="F6" s="30" t="n">
         <v>0.0006436885824909755</v>
       </c>
     </row>
@@ -29557,7 +30060,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -30153,7 +30656,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -30375,7 +30878,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -30821,7 +31324,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -30936,7 +31439,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -32512,13 +33015,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -32603,6 +33106,13 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Comisiones de las AFP (vigentes desde el 01-10-2025): SP, Sistema de AFP (spensiones.cl).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Variables macro (IPC, TPM, dólar observado, Imacec): API pública de mindicador.cl, que republica series del BCCh y el INE.</t>
         </is>

</xml_diff>